<commit_message>
Implement Sheet2 rules: OLT Type, duplicate enclosure and splitter validation, dynamic color codes, and Excel hierarchy import
</commit_message>
<xml_diff>
--- a/GPON OLT MAPPING TCR.xlsx
+++ b/GPON OLT MAPPING TCR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GPON Network Mapping Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65FF52A7-98CF-46EB-8FB9-626798CF3993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7113F883-57C0-407A-B6D3-3118EF67F1DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="216">
   <si>
     <t>Region</t>
   </si>
@@ -621,13 +621,61 @@
   </si>
   <si>
     <t>eed to capture from map</t>
+  </si>
+  <si>
+    <t>OLT Type</t>
+  </si>
+  <si>
+    <t>Can be preloaded</t>
+  </si>
+  <si>
+    <t>Drop Down 8P, 16P &amp; 32P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">for example the OLT name is " THN156 OLT53 Mulamkunnathukavu" the id should be " THN156OLT53P1E1"   Where the " THN156OLT5" is the name of the olt preloaded. P1 is the port number we do from the drop down selection and the E1 is the drop down selection from the enclosure number. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">If the Selection is 8P the drop down from P1 to P8, If the Selection is 16P the drop down from P1 to P16, If the Selection is 32P the drop down from P1 to P32 </t>
+  </si>
+  <si>
+    <t>I will upload the data from excel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drop Down From E 1 to E 20. Can not able to select the same enclosure number multiple time in a same OLT port. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drop Down S1 to S4. Can not able to select the same splitter id number under same Enclosure ID. </t>
+  </si>
+  <si>
+    <t>Splitter Lead Colour Code</t>
+  </si>
+  <si>
+    <t>ADL Subscriber ID</t>
+  </si>
+  <si>
+    <t>ACS Subscriber ID</t>
+  </si>
+  <si>
+    <t>Drop Down 1:2 , 1:4 , 1:8, 1:16 &amp; 1:32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When Select 1:2 the colour code drop down should be " 1:2 SplitterPorts 1–2: Blue, Orange " 1:4 SplitterPorts 1–4: Blue, Orange, Green, Brown"  " 1:8 SplitterPorts 1–8: Blue, Orange, Green, Brown, Slate, White, Red, Black" we will define the 1:16 &amp; 1:32 later. </t>
+  </si>
+  <si>
+    <t>Values</t>
+  </si>
+  <si>
+    <t>Type of input</t>
+  </si>
+  <si>
+    <t>Condition</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -654,8 +702,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -672,6 +726,12 @@
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -715,7 +775,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -751,6 +811,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3465,116 +3528,199 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C69B7360-1B0F-4A2F-A717-F39C3A1A3DEC}">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="255.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
         <v>1</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>2</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C2" s="12" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C3" s="12" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" s="12" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C4" s="12" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>89</v>
+        <v>3</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C5" s="12" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B8" s="12" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="C8" s="12"/>
+    </row>
+    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B9" s="12" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="C9" s="12"/>
+    </row>
+    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B10" s="12" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="C10" s="12" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B11" s="12" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="C11" s="12" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B12" s="12" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="C12" s="12"/>
+    </row>
+    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B13" s="12" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
+      <c r="C13" s="12" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B14" s="12" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
+      <c r="C14" s="12" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B15" s="12" t="s">
         <v>198</v>
       </c>
+      <c r="C15" s="12"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="C17" s="12"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="C18" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>